<commit_message>
Add Workbook-Driven Database Generation
</commit_message>
<xml_diff>
--- a/Data/Sources/EngineeringMaterials/EngineeringMaterialsDatabase.xlsx
+++ b/Data/Sources/EngineeringMaterials/EngineeringMaterialsDatabase.xlsx
@@ -2,13 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R452f159feec44a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" r:id="Rd7eeeb2b30474169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property Dictionary" sheetId="3" r:id="R1c46aa0c40cf41c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5057f212a7b64a1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPD Numeric Export" sheetId="5" r:id="R5123a10c0e664cd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selector" sheetId="6" r:id="Rfc085596d9464f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="7" r:id="R6a1a200fe51c4b0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R03d251c2d997453d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="2" r:id="R1f0ec27dded3446c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Property Dictionary" sheetId="3" r:id="Raf817399093f4386"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rac210dc86e024044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPD Numeric Export" sheetId="5" r:id="Rac00ed9b7c7b462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selector" sheetId="6" r:id="Rdec7f2ba29df4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="7" r:id="R0f2c6360e57242d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset Contract" sheetId="38" r:id="R6e76ea1bfbc34b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="39" r:id="Rebe41b8574144cd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliases" sheetId="40" r:id="Reaac0ad32e9d4c3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -29,7 +32,7 @@
     <x:numFmt numFmtId="206" formatCode="0.000E+00"/>
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -58,8 +61,19 @@
       <x:color rgb="FF17324D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos Display"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +118,61 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFDDEFE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -203,7 +272,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="53">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -323,6 +392,141 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="207" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -334,7 +538,7 @@
         <x:color rgb="FF842029"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF8D7DA"/>
         </x:patternFill>
       </x:fill>
@@ -385,8 +589,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PropertyDictionaryTable" displayName="PropertyDictionaryTable" ref="A1:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="7">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="47" name="EngineeringMaterialProperties" displayName="EngineeringMaterialProperties" ref="A1:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="Property_ID"/>
     <x:tableColumn id="2" name="CPD_Constant"/>
     <x:tableColumn id="3" name="Property_Name"/>
@@ -394,6 +598,7 @@
     <x:tableColumn id="5" name="CPD_Export_Header"/>
     <x:tableColumn id="6" name="Definition"/>
     <x:tableColumn id="7" name="Missing_Value_Behavior"/>
+    <x:tableColumn id="8" name="Materials_Source_Column"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -434,6 +639,42 @@
     <x:tableColumn id="17" name="P16_Max_Service_Temperature_C"/>
     <x:tableColumn id="18" name="P17_Hardness_HV"/>
     <x:tableColumn id="19" name="P18_Bulk_Modulus_GPa"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="44" name="EngineeringMaterialsContract" displayName="EngineeringMaterialsContract" ref="A1:C15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="Key"/>
+    <x:tableColumn id="2" name="Value"/>
+    <x:tableColumn id="3" name="Purpose"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="45" name="EngineeringMaterialCategories" displayName="EngineeringMaterialCategories" ref="A1:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Category_ID"/>
+    <x:tableColumn id="2" name="CPD_Constant"/>
+    <x:tableColumn id="3" name="Category_Name"/>
+    <x:tableColumn id="4" name="Family"/>
+    <x:tableColumn id="5" name="Category_Override"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="46" name="EngineeringMaterialAliases" displayName="EngineeringMaterialAliases" ref="A1:D193" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Alias_Type"/>
+    <x:tableColumn id="2" name="Sequence"/>
+    <x:tableColumn id="3" name="Alias_Constant"/>
+    <x:tableColumn id="4" name="Target_Constant"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -654,7 +895,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="9" t="str">
-        <x:v>Library revision</x:v>
+        <x:v>Workbook revision</x:v>
       </x:c>
       <x:c r="B3" s="10" t="str">
         <x:v>1.0.0</x:v>
@@ -662,7 +903,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
-        <x:v>Revision date</x:v>
+        <x:v>Workbook revision date</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
         <x:v>2026-08-07</x:v>
@@ -673,7 +914,7 @@
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>126 common engineering materials; 18 physical, mechanical, thermal and electrical properties</x:v>
+        <x:v>Record and populated-value counts are derived during validation and generation; no fixed count is part of the schema.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -713,7 +954,7 @@
         <x:v>Workbook relationship</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Materials is the maintainable source table; CPD Numeric Export shows the exact property-column order used by the .cpd library</x:v>
+        <x:v>Materials, Property Dictionary, Sources, Categories and Aliases are the maintained source tables; generation validates the complete workbook before atomically replacing the .cpd library.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -811,6 +1052,2726 @@
     <x:mergeCell ref="A20:F20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="37" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="98" t="str">
+        <x:v>Alias_Type</x:v>
+      </x:c>
+      <x:c r="B1" s="98" t="str">
+        <x:v>Sequence</x:v>
+      </x:c>
+      <x:c r="C1" s="98" t="str">
+        <x:v>Alias_Constant</x:v>
+      </x:c>
+      <x:c r="D1" s="98" t="str">
+        <x:v>Target_Constant</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B2" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="54" t="str">
+        <x:v>A36</x:v>
+      </x:c>
+      <x:c r="D2" s="54" t="str">
+        <x:v>STEEL_ASTM_A36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B3" s="54" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="54" t="str">
+        <x:v>STEEL_A36</x:v>
+      </x:c>
+      <x:c r="D3" s="54" t="str">
+        <x:v>STEEL_ASTM_A36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B4" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="54" t="str">
+        <x:v>AISI_1018</x:v>
+      </x:c>
+      <x:c r="D4" s="54" t="str">
+        <x:v>STEEL_AISI_1018_CD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B5" s="54" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="54" t="str">
+        <x:v>STEEL_1018</x:v>
+      </x:c>
+      <x:c r="D5" s="54" t="str">
+        <x:v>STEEL_AISI_1018_CD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B6" s="54" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C6" s="54" t="str">
+        <x:v>AISI_1020</x:v>
+      </x:c>
+      <x:c r="D6" s="54" t="str">
+        <x:v>STEEL_AISI_1020_HR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B7" s="54" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="54" t="str">
+        <x:v>STEEL_1020</x:v>
+      </x:c>
+      <x:c r="D7" s="54" t="str">
+        <x:v>STEEL_AISI_1020_HR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C8" s="54" t="str">
+        <x:v>AISI_1045</x:v>
+      </x:c>
+      <x:c r="D8" s="54" t="str">
+        <x:v>STEEL_AISI_1045_N</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B9" s="54" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" s="54" t="str">
+        <x:v>STEEL_1045</x:v>
+      </x:c>
+      <x:c r="D9" s="54" t="str">
+        <x:v>STEEL_AISI_1045_N</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B10" s="54" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C10" s="54" t="str">
+        <x:v>AISI_1095</x:v>
+      </x:c>
+      <x:c r="D10" s="54" t="str">
+        <x:v>STEEL_AISI_1095_A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B11" s="54" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C11" s="54" t="str">
+        <x:v>STEEL_1095</x:v>
+      </x:c>
+      <x:c r="D11" s="54" t="str">
+        <x:v>STEEL_AISI_1095_A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B12" s="54" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C12" s="54" t="str">
+        <x:v>AISI_4130</x:v>
+      </x:c>
+      <x:c r="D12" s="54" t="str">
+        <x:v>STEEL_AISI_4130_N</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B13" s="54" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C13" s="54" t="str">
+        <x:v>STEEL_4130</x:v>
+      </x:c>
+      <x:c r="D13" s="54" t="str">
+        <x:v>STEEL_AISI_4130_N</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B14" s="54" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C14" s="54" t="str">
+        <x:v>AISI_4140</x:v>
+      </x:c>
+      <x:c r="D14" s="54" t="str">
+        <x:v>STEEL_AISI_4140_QT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C15" s="54" t="str">
+        <x:v>STEEL_4140</x:v>
+      </x:c>
+      <x:c r="D15" s="54" t="str">
+        <x:v>STEEL_AISI_4140_QT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B16" s="54" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C16" s="54" t="str">
+        <x:v>AISI_4340</x:v>
+      </x:c>
+      <x:c r="D16" s="54" t="str">
+        <x:v>STEEL_AISI_4340_QT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B17" s="54" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C17" s="54" t="str">
+        <x:v>STEEL_4340</x:v>
+      </x:c>
+      <x:c r="D17" s="54" t="str">
+        <x:v>STEEL_AISI_4340_QT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B18" s="54" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C18" s="54" t="str">
+        <x:v>A572_GR50</x:v>
+      </x:c>
+      <x:c r="D18" s="54" t="str">
+        <x:v>STEEL_ASTM_A572_GR50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B19" s="54" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C19" s="54" t="str">
+        <x:v>STEEL_A572_GR50</x:v>
+      </x:c>
+      <x:c r="D19" s="54" t="str">
+        <x:v>STEEL_ASTM_A572_GR50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B20" s="54" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C20" s="54" t="str">
+        <x:v>A992</x:v>
+      </x:c>
+      <x:c r="D20" s="54" t="str">
+        <x:v>STEEL_ASTM_A992</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B21" s="54" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C21" s="54" t="str">
+        <x:v>STEEL_A992</x:v>
+      </x:c>
+      <x:c r="D21" s="54" t="str">
+        <x:v>STEEL_ASTM_A992</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B22" s="54" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C22" s="54" t="str">
+        <x:v>TOOL_STEEL_A2</x:v>
+      </x:c>
+      <x:c r="D22" s="54" t="str">
+        <x:v>TOOL_STEEL_A2_HARDENED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B23" s="54" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="C23" s="54" t="str">
+        <x:v>TOOL_STEEL_D2</x:v>
+      </x:c>
+      <x:c r="D23" s="54" t="str">
+        <x:v>TOOL_STEEL_D2_HARDENED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B24" s="54" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C24" s="54" t="str">
+        <x:v>TOOL_STEEL_H13</x:v>
+      </x:c>
+      <x:c r="D24" s="54" t="str">
+        <x:v>TOOL_STEEL_H13_HARDENED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B25" s="54" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C25" s="54" t="str">
+        <x:v>MARAGING_250</x:v>
+      </x:c>
+      <x:c r="D25" s="54" t="str">
+        <x:v>MARAGING_STEEL_18NI_250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B26" s="54" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C26" s="54" t="str">
+        <x:v>SS304</x:v>
+      </x:c>
+      <x:c r="D26" s="54" t="str">
+        <x:v>STAINLESS_304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B27" s="54" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="C27" s="54" t="str">
+        <x:v>AISI_304</x:v>
+      </x:c>
+      <x:c r="D27" s="54" t="str">
+        <x:v>STAINLESS_304</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B28" s="54" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="C28" s="54" t="str">
+        <x:v>SS304L</x:v>
+      </x:c>
+      <x:c r="D28" s="54" t="str">
+        <x:v>STAINLESS_304L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B29" s="54" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C29" s="54" t="str">
+        <x:v>AISI_304L</x:v>
+      </x:c>
+      <x:c r="D29" s="54" t="str">
+        <x:v>STAINLESS_304L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B30" s="54" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C30" s="54" t="str">
+        <x:v>SS316</x:v>
+      </x:c>
+      <x:c r="D30" s="54" t="str">
+        <x:v>STAINLESS_316</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B31" s="54" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="C31" s="54" t="str">
+        <x:v>AISI_316</x:v>
+      </x:c>
+      <x:c r="D31" s="54" t="str">
+        <x:v>STAINLESS_316</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B32" s="54" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C32" s="54" t="str">
+        <x:v>SS316L</x:v>
+      </x:c>
+      <x:c r="D32" s="54" t="str">
+        <x:v>STAINLESS_316L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B33" s="54" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C33" s="54" t="str">
+        <x:v>AISI_316L</x:v>
+      </x:c>
+      <x:c r="D33" s="54" t="str">
+        <x:v>STAINLESS_316L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B34" s="54" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="C34" s="54" t="str">
+        <x:v>SS321</x:v>
+      </x:c>
+      <x:c r="D34" s="54" t="str">
+        <x:v>STAINLESS_321</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B35" s="54" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C35" s="54" t="str">
+        <x:v>AISI_321</x:v>
+      </x:c>
+      <x:c r="D35" s="54" t="str">
+        <x:v>STAINLESS_321</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B36" s="54" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C36" s="54" t="str">
+        <x:v>SS410</x:v>
+      </x:c>
+      <x:c r="D36" s="54" t="str">
+        <x:v>STAINLESS_410_A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B37" s="54" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="C37" s="54" t="str">
+        <x:v>AISI_410</x:v>
+      </x:c>
+      <x:c r="D37" s="54" t="str">
+        <x:v>STAINLESS_410_A</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B38" s="54" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="C38" s="54" t="str">
+        <x:v>SS420</x:v>
+      </x:c>
+      <x:c r="D38" s="54" t="str">
+        <x:v>STAINLESS_420_H</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B39" s="54" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C39" s="54" t="str">
+        <x:v>AISI_420</x:v>
+      </x:c>
+      <x:c r="D39" s="54" t="str">
+        <x:v>STAINLESS_420_H</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B40" s="54" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C40" s="54" t="str">
+        <x:v>SS430</x:v>
+      </x:c>
+      <x:c r="D40" s="54" t="str">
+        <x:v>STAINLESS_430</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B41" s="54" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C41" s="54" t="str">
+        <x:v>AISI_430</x:v>
+      </x:c>
+      <x:c r="D41" s="54" t="str">
+        <x:v>STAINLESS_430</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B42" s="54" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="C42" s="54" t="str">
+        <x:v>SS17_4PH</x:v>
+      </x:c>
+      <x:c r="D42" s="54" t="str">
+        <x:v>STAINLESS_17_4PH_H900</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B43" s="54" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="C43" s="54" t="str">
+        <x:v>DUPLEX_2205</x:v>
+      </x:c>
+      <x:c r="D43" s="54" t="str">
+        <x:v>STAINLESS_DUPLEX_2205</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B44" s="54" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C44" s="54" t="str">
+        <x:v>SS2205</x:v>
+      </x:c>
+      <x:c r="D44" s="54" t="str">
+        <x:v>STAINLESS_DUPLEX_2205</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B45" s="54" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="C45" s="54" t="str">
+        <x:v>GRAY_IRON_CLASS_30</x:v>
+      </x:c>
+      <x:c r="D45" s="54" t="str">
+        <x:v>CAST_IRON_GRAY_CLASS_30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B46" s="54" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="C46" s="54" t="str">
+        <x:v>DUCTILE_IRON_65_45_12</x:v>
+      </x:c>
+      <x:c r="D46" s="54" t="str">
+        <x:v>CAST_IRON_DUCTILE_65_45_12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B47" s="54" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="C47" s="54" t="str">
+        <x:v>CGI_CAST_IRON</x:v>
+      </x:c>
+      <x:c r="D47" s="54" t="str">
+        <x:v>CAST_IRON_COMPACTED_GRAPHITE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B48" s="54" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C48" s="54" t="str">
+        <x:v>AL1100_H14</x:v>
+      </x:c>
+      <x:c r="D48" s="54" t="str">
+        <x:v>ALUMINUM_1100_H14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B49" s="54" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="C49" s="54" t="str">
+        <x:v>AL2024_T3</x:v>
+      </x:c>
+      <x:c r="D49" s="54" t="str">
+        <x:v>ALUMINUM_2024_T3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B50" s="54" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="C50" s="54" t="str">
+        <x:v>AL3003_H14</x:v>
+      </x:c>
+      <x:c r="D50" s="54" t="str">
+        <x:v>ALUMINUM_3003_H14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B51" s="54" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C51" s="54" t="str">
+        <x:v>AL5052_H32</x:v>
+      </x:c>
+      <x:c r="D51" s="54" t="str">
+        <x:v>ALUMINUM_5052_H32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B52" s="54" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C52" s="54" t="str">
+        <x:v>AL5083_H116</x:v>
+      </x:c>
+      <x:c r="D52" s="54" t="str">
+        <x:v>ALUMINUM_5083_H116</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B53" s="54" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="C53" s="54" t="str">
+        <x:v>AL6061_T6</x:v>
+      </x:c>
+      <x:c r="D53" s="54" t="str">
+        <x:v>ALUMINUM_6061_T6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B54" s="54" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="C54" s="54" t="str">
+        <x:v>ALUMINUM_6061</x:v>
+      </x:c>
+      <x:c r="D54" s="54" t="str">
+        <x:v>ALUMINUM_6061_T6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B55" s="54" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C55" s="54" t="str">
+        <x:v>AL6063_T5</x:v>
+      </x:c>
+      <x:c r="D55" s="54" t="str">
+        <x:v>ALUMINUM_6063_T5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B56" s="54" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C56" s="54" t="str">
+        <x:v>AL7075_T6</x:v>
+      </x:c>
+      <x:c r="D56" s="54" t="str">
+        <x:v>ALUMINUM_7075_T6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B57" s="54" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C57" s="54" t="str">
+        <x:v>A356_T6</x:v>
+      </x:c>
+      <x:c r="D57" s="54" t="str">
+        <x:v>ALUMINUM_A356_T6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B58" s="54" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C58" s="54" t="str">
+        <x:v>COPPER_C110</x:v>
+      </x:c>
+      <x:c r="D58" s="54" t="str">
+        <x:v>COPPER_C110_ANNEALED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B59" s="54" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="C59" s="54" t="str">
+        <x:v>C110_COPPER</x:v>
+      </x:c>
+      <x:c r="D59" s="54" t="str">
+        <x:v>COPPER_C110_ANNEALED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B60" s="54" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C60" s="54" t="str">
+        <x:v>BRASS_C260</x:v>
+      </x:c>
+      <x:c r="D60" s="54" t="str">
+        <x:v>BRASS_C260_H02</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B61" s="54" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C61" s="54" t="str">
+        <x:v>BRONZE_C510</x:v>
+      </x:c>
+      <x:c r="D61" s="54" t="str">
+        <x:v>PHOSPHOR_BRONZE_C510</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B62" s="54" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C62" s="54" t="str">
+        <x:v>BRONZE_C932</x:v>
+      </x:c>
+      <x:c r="D62" s="54" t="str">
+        <x:v>BEARING_BRONZE_C932</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B63" s="54" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C63" s="54" t="str">
+        <x:v>C715_COPPER_NICKEL</x:v>
+      </x:c>
+      <x:c r="D63" s="54" t="str">
+        <x:v>COPPER_NICKEL_C715</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B64" s="54" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C64" s="54" t="str">
+        <x:v>CUNi_70_30</x:v>
+      </x:c>
+      <x:c r="D64" s="54" t="str">
+        <x:v>COPPER_NICKEL_C715</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B65" s="54" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C65" s="54" t="str">
+        <x:v>MG_AZ31B</x:v>
+      </x:c>
+      <x:c r="D65" s="54" t="str">
+        <x:v>MAGNESIUM_AZ31B_H24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B66" s="54" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="C66" s="54" t="str">
+        <x:v>MG_AZ91D</x:v>
+      </x:c>
+      <x:c r="D66" s="54" t="str">
+        <x:v>MAGNESIUM_AZ91D_T6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B67" s="54" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C67" s="54" t="str">
+        <x:v>TI_GRADE_2</x:v>
+      </x:c>
+      <x:c r="D67" s="54" t="str">
+        <x:v>TITANIUM_GRADE_2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B68" s="54" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C68" s="54" t="str">
+        <x:v>TI6AL4V</x:v>
+      </x:c>
+      <x:c r="D68" s="54" t="str">
+        <x:v>TITANIUM_TI6AL4V_ANNEALED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B69" s="54" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C69" s="54" t="str">
+        <x:v>TITANIUM_GRADE_5</x:v>
+      </x:c>
+      <x:c r="D69" s="54" t="str">
+        <x:v>TITANIUM_TI6AL4V_ANNEALED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B70" s="54" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="C70" s="54" t="str">
+        <x:v>NI200</x:v>
+      </x:c>
+      <x:c r="D70" s="54" t="str">
+        <x:v>NICKEL_200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B71" s="54" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C71" s="54" t="str">
+        <x:v>NICKEL200</x:v>
+      </x:c>
+      <x:c r="D71" s="54" t="str">
+        <x:v>NICKEL_200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B72" s="54" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="C72" s="54" t="str">
+        <x:v>MONEL400</x:v>
+      </x:c>
+      <x:c r="D72" s="54" t="str">
+        <x:v>MONEL_400</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B73" s="54" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C73" s="54" t="str">
+        <x:v>INCONEL625</x:v>
+      </x:c>
+      <x:c r="D73" s="54" t="str">
+        <x:v>INCONEL_625</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B74" s="54" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="C74" s="54" t="str">
+        <x:v>INCONEL718</x:v>
+      </x:c>
+      <x:c r="D74" s="54" t="str">
+        <x:v>INCONEL_718_AGED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B75" s="54" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="C75" s="54" t="str">
+        <x:v>C276</x:v>
+      </x:c>
+      <x:c r="D75" s="54" t="str">
+        <x:v>HASTELLOY_C276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B76" s="54" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C76" s="54" t="str">
+        <x:v>HASTELLOY_C_276</x:v>
+      </x:c>
+      <x:c r="D76" s="54" t="str">
+        <x:v>HASTELLOY_C276</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B77" s="54" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C77" s="54" t="str">
+        <x:v>ZAMAK3</x:v>
+      </x:c>
+      <x:c r="D77" s="54" t="str">
+        <x:v>ZINC_ZAMAK_3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B78" s="54" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="C78" s="54" t="str">
+        <x:v>LEAD</x:v>
+      </x:c>
+      <x:c r="D78" s="54" t="str">
+        <x:v>LEAD_PURE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B79" s="54" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C79" s="54" t="str">
+        <x:v>TIN</x:v>
+      </x:c>
+      <x:c r="D79" s="54" t="str">
+        <x:v>TIN_PURE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B80" s="54" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C80" s="54" t="str">
+        <x:v>ABS</x:v>
+      </x:c>
+      <x:c r="D80" s="54" t="str">
+        <x:v>POLYMER_ABS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B81" s="54" t="n">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="C81" s="54" t="str">
+        <x:v>PLA</x:v>
+      </x:c>
+      <x:c r="D81" s="54" t="str">
+        <x:v>POLYMER_PLA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B82" s="54" t="n">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="C82" s="54" t="str">
+        <x:v>HIPS</x:v>
+      </x:c>
+      <x:c r="D82" s="54" t="str">
+        <x:v>POLYMER_HIPS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B83" s="54" t="n">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C83" s="54" t="str">
+        <x:v>HDPE</x:v>
+      </x:c>
+      <x:c r="D83" s="54" t="str">
+        <x:v>POLYMER_HDPE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B84" s="54" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="C84" s="54" t="str">
+        <x:v>LDPE</x:v>
+      </x:c>
+      <x:c r="D84" s="54" t="str">
+        <x:v>POLYMER_LDPE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B85" s="54" t="n">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="C85" s="54" t="str">
+        <x:v>UHMWPE</x:v>
+      </x:c>
+      <x:c r="D85" s="54" t="str">
+        <x:v>POLYMER_UHMWPE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B86" s="54" t="n">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="C86" s="54" t="str">
+        <x:v>PP</x:v>
+      </x:c>
+      <x:c r="D86" s="54" t="str">
+        <x:v>POLYMER_PP_HOMOPOLYMER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B87" s="54" t="n">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="C87" s="54" t="str">
+        <x:v>POLYPROPYLENE</x:v>
+      </x:c>
+      <x:c r="D87" s="54" t="str">
+        <x:v>POLYMER_PP_HOMOPOLYMER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B88" s="54" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C88" s="54" t="str">
+        <x:v>PVC</x:v>
+      </x:c>
+      <x:c r="D88" s="54" t="str">
+        <x:v>POLYMER_PVC_RIGID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B89" s="54" t="n">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="C89" s="54" t="str">
+        <x:v>UPVC</x:v>
+      </x:c>
+      <x:c r="D89" s="54" t="str">
+        <x:v>POLYMER_PVC_RIGID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B90" s="54" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="C90" s="54" t="str">
+        <x:v>CPVC</x:v>
+      </x:c>
+      <x:c r="D90" s="54" t="str">
+        <x:v>POLYMER_CPVC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B91" s="54" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C91" s="54" t="str">
+        <x:v>PET</x:v>
+      </x:c>
+      <x:c r="D91" s="54" t="str">
+        <x:v>POLYMER_PET</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B92" s="54" t="n">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C92" s="54" t="str">
+        <x:v>PETG</x:v>
+      </x:c>
+      <x:c r="D92" s="54" t="str">
+        <x:v>POLYMER_PETG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B93" s="54" t="n">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="C93" s="54" t="str">
+        <x:v>PA6</x:v>
+      </x:c>
+      <x:c r="D93" s="54" t="str">
+        <x:v>POLYMER_PA6_DRY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B94" s="54" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="C94" s="54" t="str">
+        <x:v>NYLON6</x:v>
+      </x:c>
+      <x:c r="D94" s="54" t="str">
+        <x:v>POLYMER_PA6_DRY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B95" s="54" t="n">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="C95" s="54" t="str">
+        <x:v>PA66</x:v>
+      </x:c>
+      <x:c r="D95" s="54" t="str">
+        <x:v>POLYMER_PA66_DRY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B96" s="54" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="C96" s="54" t="str">
+        <x:v>NYLON66</x:v>
+      </x:c>
+      <x:c r="D96" s="54" t="str">
+        <x:v>POLYMER_PA66_DRY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B97" s="54" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C97" s="54" t="str">
+        <x:v>POM</x:v>
+      </x:c>
+      <x:c r="D97" s="54" t="str">
+        <x:v>POLYMER_POM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B98" s="54" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="C98" s="54" t="str">
+        <x:v>ACETAL</x:v>
+      </x:c>
+      <x:c r="D98" s="54" t="str">
+        <x:v>POLYMER_POM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B99" s="54" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C99" s="54" t="str">
+        <x:v>PC</x:v>
+      </x:c>
+      <x:c r="D99" s="54" t="str">
+        <x:v>POLYMER_PC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B100" s="54" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C100" s="54" t="str">
+        <x:v>POLYCARBONATE</x:v>
+      </x:c>
+      <x:c r="D100" s="54" t="str">
+        <x:v>POLYMER_PC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B101" s="54" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="C101" s="54" t="str">
+        <x:v>PMMA</x:v>
+      </x:c>
+      <x:c r="D101" s="54" t="str">
+        <x:v>POLYMER_PMMA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B102" s="54" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="C102" s="54" t="str">
+        <x:v>ACRYLIC</x:v>
+      </x:c>
+      <x:c r="D102" s="54" t="str">
+        <x:v>POLYMER_PMMA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B103" s="54" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="C103" s="54" t="str">
+        <x:v>PTFE</x:v>
+      </x:c>
+      <x:c r="D103" s="54" t="str">
+        <x:v>POLYMER_PTFE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B104" s="54" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="C104" s="54" t="str">
+        <x:v>TEFLON</x:v>
+      </x:c>
+      <x:c r="D104" s="54" t="str">
+        <x:v>POLYMER_PTFE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B105" s="54" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C105" s="54" t="str">
+        <x:v>PEEK</x:v>
+      </x:c>
+      <x:c r="D105" s="54" t="str">
+        <x:v>POLYMER_PEEK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B106" s="54" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="C106" s="54" t="str">
+        <x:v>PEI</x:v>
+      </x:c>
+      <x:c r="D106" s="54" t="str">
+        <x:v>POLYMER_PEI</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B107" s="54" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="C107" s="54" t="str">
+        <x:v>PPS</x:v>
+      </x:c>
+      <x:c r="D107" s="54" t="str">
+        <x:v>POLYMER_PPS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B108" s="54" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="C108" s="54" t="str">
+        <x:v>PSU</x:v>
+      </x:c>
+      <x:c r="D108" s="54" t="str">
+        <x:v>POLYMER_PSU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B109" s="54" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C109" s="54" t="str">
+        <x:v>POLYSULFONE</x:v>
+      </x:c>
+      <x:c r="D109" s="54" t="str">
+        <x:v>POLYMER_PSU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B110" s="54" t="n">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="C110" s="54" t="str">
+        <x:v>EPOXY</x:v>
+      </x:c>
+      <x:c r="D110" s="54" t="str">
+        <x:v>POLYMER_EPOXY_CAST</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B111" s="54" t="n">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="C111" s="54" t="str">
+        <x:v>PHENOLIC</x:v>
+      </x:c>
+      <x:c r="D111" s="54" t="str">
+        <x:v>POLYMER_PHENOLIC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B112" s="54" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="C112" s="54" t="str">
+        <x:v>PBT</x:v>
+      </x:c>
+      <x:c r="D112" s="54" t="str">
+        <x:v>POLYMER_PBT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B113" s="54" t="n">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="C113" s="54" t="str">
+        <x:v>PVDF</x:v>
+      </x:c>
+      <x:c r="D113" s="54" t="str">
+        <x:v>POLYMER_PVDF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B114" s="54" t="n">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C114" s="54" t="str">
+        <x:v>NATURAL_RUBBER</x:v>
+      </x:c>
+      <x:c r="D114" s="54" t="str">
+        <x:v>ELASTOMER_NATURAL_RUBBER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B115" s="54" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="C115" s="54" t="str">
+        <x:v>NR_RUBBER</x:v>
+      </x:c>
+      <x:c r="D115" s="54" t="str">
+        <x:v>ELASTOMER_NATURAL_RUBBER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B116" s="54" t="n">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="C116" s="54" t="str">
+        <x:v>NEOPRENE</x:v>
+      </x:c>
+      <x:c r="D116" s="54" t="str">
+        <x:v>ELASTOMER_NEOPRENE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B117" s="54" t="n">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="C117" s="54" t="str">
+        <x:v>CR_RUBBER</x:v>
+      </x:c>
+      <x:c r="D117" s="54" t="str">
+        <x:v>ELASTOMER_NEOPRENE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B118" s="54" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="C118" s="54" t="str">
+        <x:v>NBR</x:v>
+      </x:c>
+      <x:c r="D118" s="54" t="str">
+        <x:v>ELASTOMER_NBR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B119" s="54" t="n">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="C119" s="54" t="str">
+        <x:v>NITRILE_RUBBER</x:v>
+      </x:c>
+      <x:c r="D119" s="54" t="str">
+        <x:v>ELASTOMER_NBR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B120" s="54" t="n">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C120" s="54" t="str">
+        <x:v>EPDM</x:v>
+      </x:c>
+      <x:c r="D120" s="54" t="str">
+        <x:v>ELASTOMER_EPDM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B121" s="54" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C121" s="54" t="str">
+        <x:v>SILICONE_RUBBER</x:v>
+      </x:c>
+      <x:c r="D121" s="54" t="str">
+        <x:v>ELASTOMER_SILICONE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B122" s="54" t="n">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="C122" s="54" t="str">
+        <x:v>FKM</x:v>
+      </x:c>
+      <x:c r="D122" s="54" t="str">
+        <x:v>ELASTOMER_FKM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B123" s="54" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C123" s="54" t="str">
+        <x:v>FLUOROELASTOMER</x:v>
+      </x:c>
+      <x:c r="D123" s="54" t="str">
+        <x:v>ELASTOMER_FKM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B124" s="54" t="n">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="C124" s="54" t="str">
+        <x:v>TPU</x:v>
+      </x:c>
+      <x:c r="D124" s="54" t="str">
+        <x:v>ELASTOMER_TPU</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B125" s="54" t="n">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="C125" s="54" t="str">
+        <x:v>SODA_LIME_GLASS</x:v>
+      </x:c>
+      <x:c r="D125" s="54" t="str">
+        <x:v>GLASS_SODA_LIME</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B126" s="54" t="n">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C126" s="54" t="str">
+        <x:v>BOROSILICATE_GLASS</x:v>
+      </x:c>
+      <x:c r="D126" s="54" t="str">
+        <x:v>GLASS_BOROSILICATE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B127" s="54" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C127" s="54" t="str">
+        <x:v>FUSED_SILICA</x:v>
+      </x:c>
+      <x:c r="D127" s="54" t="str">
+        <x:v>GLASS_FUSED_SILICA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B128" s="54" t="n">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="C128" s="54" t="str">
+        <x:v>ALUMINA_96</x:v>
+      </x:c>
+      <x:c r="D128" s="54" t="str">
+        <x:v>CERAMIC_ALUMINA_96</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B129" s="54" t="n">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C129" s="54" t="str">
+        <x:v>ALUMINA_995</x:v>
+      </x:c>
+      <x:c r="D129" s="54" t="str">
+        <x:v>CERAMIC_ALUMINA_995</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B130" s="54" t="n">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="C130" s="54" t="str">
+        <x:v>YTZP</x:v>
+      </x:c>
+      <x:c r="D130" s="54" t="str">
+        <x:v>CERAMIC_ZIRCONIA_YTZP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B131" s="54" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="C131" s="54" t="str">
+        <x:v>ZIRCONIA_YTZP</x:v>
+      </x:c>
+      <x:c r="D131" s="54" t="str">
+        <x:v>CERAMIC_ZIRCONIA_YTZP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B132" s="54" t="n">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="C132" s="54" t="str">
+        <x:v>SILICON_CARBIDE</x:v>
+      </x:c>
+      <x:c r="D132" s="54" t="str">
+        <x:v>CERAMIC_SILICON_CARBIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B133" s="54" t="n">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="C133" s="54" t="str">
+        <x:v>SIC</x:v>
+      </x:c>
+      <x:c r="D133" s="54" t="str">
+        <x:v>CERAMIC_SILICON_CARBIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B134" s="54" t="n">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="C134" s="54" t="str">
+        <x:v>SILICON_NITRIDE</x:v>
+      </x:c>
+      <x:c r="D134" s="54" t="str">
+        <x:v>CERAMIC_SILICON_NITRIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B135" s="54" t="n">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="C135" s="54" t="str">
+        <x:v>SI3N4</x:v>
+      </x:c>
+      <x:c r="D135" s="54" t="str">
+        <x:v>CERAMIC_SILICON_NITRIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B136" s="54" t="n">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="C136" s="54" t="str">
+        <x:v>ALUMINUM_NITRIDE</x:v>
+      </x:c>
+      <x:c r="D136" s="54" t="str">
+        <x:v>CERAMIC_ALUMINUM_NITRIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B137" s="54" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C137" s="54" t="str">
+        <x:v>ALN</x:v>
+      </x:c>
+      <x:c r="D137" s="54" t="str">
+        <x:v>CERAMIC_ALUMINUM_NITRIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B138" s="54" t="n">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="C138" s="54" t="str">
+        <x:v>BORON_CARBIDE</x:v>
+      </x:c>
+      <x:c r="D138" s="54" t="str">
+        <x:v>CERAMIC_BORON_CARBIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B139" s="54" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="C139" s="54" t="str">
+        <x:v>B4C</x:v>
+      </x:c>
+      <x:c r="D139" s="54" t="str">
+        <x:v>CERAMIC_BORON_CARBIDE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B140" s="54" t="n">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="C140" s="54" t="str">
+        <x:v>MULLITE</x:v>
+      </x:c>
+      <x:c r="D140" s="54" t="str">
+        <x:v>CERAMIC_MULLITE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B141" s="54" t="n">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="C141" s="54" t="str">
+        <x:v>ELECTRICAL_PORCELAIN</x:v>
+      </x:c>
+      <x:c r="D141" s="54" t="str">
+        <x:v>CERAMIC_PORCELAIN_ELECTRICAL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B142" s="54" t="n">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="C142" s="54" t="str">
+        <x:v>GRAPHITE</x:v>
+      </x:c>
+      <x:c r="D142" s="54" t="str">
+        <x:v>CARBON_GRAPHITE_ISOTROPIC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B143" s="54" t="n">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="C143" s="54" t="str">
+        <x:v>WC_6CO</x:v>
+      </x:c>
+      <x:c r="D143" s="54" t="str">
+        <x:v>CERMET_TUNGSTEN_CARBIDE_6CO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B144" s="54" t="n">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C144" s="54" t="str">
+        <x:v>TUNGSTEN_CARBIDE</x:v>
+      </x:c>
+      <x:c r="D144" s="54" t="str">
+        <x:v>CERMET_TUNGSTEN_CARBIDE_6CO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B145" s="54" t="n">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="C145" s="54" t="str">
+        <x:v>STEATITE</x:v>
+      </x:c>
+      <x:c r="D145" s="54" t="str">
+        <x:v>CERAMIC_STEATITE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B146" s="54" t="n">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="C146" s="54" t="str">
+        <x:v>CORDIERITE</x:v>
+      </x:c>
+      <x:c r="D146" s="54" t="str">
+        <x:v>CERAMIC_CORDIERITE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B147" s="54" t="n">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="C147" s="54" t="str">
+        <x:v>CFRP_UD</x:v>
+      </x:c>
+      <x:c r="D147" s="54" t="str">
+        <x:v>COMPOSITE_CFRP_UD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B148" s="54" t="n">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="C148" s="54" t="str">
+        <x:v>CFRP_QUASI</x:v>
+      </x:c>
+      <x:c r="D148" s="54" t="str">
+        <x:v>COMPOSITE_CFRP_QUASI_ISO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B149" s="54" t="n">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="C149" s="54" t="str">
+        <x:v>GFRP_UD</x:v>
+      </x:c>
+      <x:c r="D149" s="54" t="str">
+        <x:v>COMPOSITE_GFRP_UD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B150" s="54" t="n">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="C150" s="54" t="str">
+        <x:v>GFRP_QUASI</x:v>
+      </x:c>
+      <x:c r="D150" s="54" t="str">
+        <x:v>COMPOSITE_GFRP_QUASI_ISO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B151" s="54" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C151" s="54" t="str">
+        <x:v>ARAMID_EPOXY_UD</x:v>
+      </x:c>
+      <x:c r="D151" s="54" t="str">
+        <x:v>COMPOSITE_ARAMID_EPOXY_UD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B152" s="54" t="n">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="C152" s="54" t="str">
+        <x:v>KEVLAR_EPOXY_UD</x:v>
+      </x:c>
+      <x:c r="D152" s="54" t="str">
+        <x:v>COMPOSITE_ARAMID_EPOXY_UD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B153" s="54" t="n">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="C153" s="54" t="str">
+        <x:v>DOUGLAS_FIR</x:v>
+      </x:c>
+      <x:c r="D153" s="54" t="str">
+        <x:v>WOOD_DOUGLAS_FIR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B154" s="54" t="n">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="C154" s="54" t="str">
+        <x:v>SPF_WOOD</x:v>
+      </x:c>
+      <x:c r="D154" s="54" t="str">
+        <x:v>WOOD_SPRUCE_PINE_FIR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B155" s="54" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="C155" s="54" t="str">
+        <x:v>SOUTHERN_PINE</x:v>
+      </x:c>
+      <x:c r="D155" s="54" t="str">
+        <x:v>WOOD_SOUTHERN_PINE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B156" s="54" t="n">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="C156" s="54" t="str">
+        <x:v>WHITE_OAK</x:v>
+      </x:c>
+      <x:c r="D156" s="54" t="str">
+        <x:v>WOOD_WHITE_OAK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B157" s="54" t="n">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="C157" s="54" t="str">
+        <x:v>HARD_MAPLE</x:v>
+      </x:c>
+      <x:c r="D157" s="54" t="str">
+        <x:v>WOOD_HARD_MAPLE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B158" s="54" t="n">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="C158" s="54" t="str">
+        <x:v>SOFTWOOD_PLYWOOD</x:v>
+      </x:c>
+      <x:c r="D158" s="54" t="str">
+        <x:v>WOOD_PLYWOOD_SOFTWOOD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B159" s="54" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="C159" s="54" t="str">
+        <x:v>PLYWOOD</x:v>
+      </x:c>
+      <x:c r="D159" s="54" t="str">
+        <x:v>WOOD_PLYWOOD_SOFTWOOD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B160" s="54" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="C160" s="54" t="str">
+        <x:v>MDF</x:v>
+      </x:c>
+      <x:c r="D160" s="54" t="str">
+        <x:v>WOOD_MDF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B161" s="54" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="C161" s="54" t="str">
+        <x:v>LVL</x:v>
+      </x:c>
+      <x:c r="D161" s="54" t="str">
+        <x:v>WOOD_LVL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B162" s="54" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C162" s="54" t="str">
+        <x:v>GLULAM</x:v>
+      </x:c>
+      <x:c r="D162" s="54" t="str">
+        <x:v>WOOD_GLULAM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B163" s="54" t="n">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C163" s="54" t="str">
+        <x:v>CONCRETE_25MPA</x:v>
+      </x:c>
+      <x:c r="D163" s="54" t="str">
+        <x:v>CONCRETE_NORMAL_25MPA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B164" s="54" t="n">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C164" s="54" t="str">
+        <x:v>CONCRETE_40MPA</x:v>
+      </x:c>
+      <x:c r="D164" s="54" t="str">
+        <x:v>CONCRETE_NORMAL_40MPA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B165" s="54" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="C165" s="54" t="str">
+        <x:v>CONCRETE_60MPA</x:v>
+      </x:c>
+      <x:c r="D165" s="54" t="str">
+        <x:v>CONCRETE_NORMAL_60MPA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B166" s="54" t="n">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="C166" s="54" t="str">
+        <x:v>LIGHTWEIGHT_CONCRETE</x:v>
+      </x:c>
+      <x:c r="D166" s="54" t="str">
+        <x:v>CONCRETE_LIGHTWEIGHT_25MPA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B167" s="54" t="n">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="C167" s="54" t="str">
+        <x:v>CLAY_BRICK</x:v>
+      </x:c>
+      <x:c r="D167" s="54" t="str">
+        <x:v>MASONRY_FIRED_CLAY_BRICK</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B168" s="54" t="n">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="C168" s="54" t="str">
+        <x:v>GRANITE</x:v>
+      </x:c>
+      <x:c r="D168" s="54" t="str">
+        <x:v>STONE_GRANITE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B169" s="54" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="C169" s="54" t="str">
+        <x:v>LIMESTONE</x:v>
+      </x:c>
+      <x:c r="D169" s="54" t="str">
+        <x:v>STONE_LIMESTONE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B170" s="54" t="n">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="C170" s="54" t="str">
+        <x:v>SANDSTONE</x:v>
+      </x:c>
+      <x:c r="D170" s="54" t="str">
+        <x:v>STONE_SANDSTONE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B171" s="54" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="C171" s="54" t="str">
+        <x:v>DRYWALL</x:v>
+      </x:c>
+      <x:c r="D171" s="54" t="str">
+        <x:v>GYPSUM_BOARD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B172" s="54" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="C172" s="54" t="str">
+        <x:v>GYPSUM_WALLBOARD</x:v>
+      </x:c>
+      <x:c r="D172" s="54" t="str">
+        <x:v>GYPSUM_BOARD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="54" t="str">
+        <x:v>Material</x:v>
+      </x:c>
+      <x:c r="B173" s="54" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="C173" s="54" t="str">
+        <x:v>ASPHALT</x:v>
+      </x:c>
+      <x:c r="D173" s="54" t="str">
+        <x:v>ASPHALT_CONCRETE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B174" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C174" s="54" t="str">
+        <x:v>MAT_DENSITY</x:v>
+      </x:c>
+      <x:c r="D174" s="54" t="str">
+        <x:v>MAT_P_DENSITY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B175" s="54" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C175" s="54" t="str">
+        <x:v>MAT_RHO</x:v>
+      </x:c>
+      <x:c r="D175" s="54" t="str">
+        <x:v>MAT_P_DENSITY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B176" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C176" s="54" t="str">
+        <x:v>MAT_E</x:v>
+      </x:c>
+      <x:c r="D176" s="54" t="str">
+        <x:v>MAT_P_YOUNGS_MODULUS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B177" s="54" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C177" s="54" t="str">
+        <x:v>MAT_ELASTIC_MODULUS</x:v>
+      </x:c>
+      <x:c r="D177" s="54" t="str">
+        <x:v>MAT_P_YOUNGS_MODULUS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B178" s="54" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C178" s="54" t="str">
+        <x:v>MAT_G</x:v>
+      </x:c>
+      <x:c r="D178" s="54" t="str">
+        <x:v>MAT_P_SHEAR_MODULUS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B179" s="54" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C179" s="54" t="str">
+        <x:v>MAT_NU</x:v>
+      </x:c>
+      <x:c r="D179" s="54" t="str">
+        <x:v>MAT_P_POISSON_RATIO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B180" s="54" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C180" s="54" t="str">
+        <x:v>MAT_YIELD</x:v>
+      </x:c>
+      <x:c r="D180" s="54" t="str">
+        <x:v>MAT_P_YIELD_STRENGTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B181" s="54" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C181" s="54" t="str">
+        <x:v>MAT_UTS</x:v>
+      </x:c>
+      <x:c r="D181" s="54" t="str">
+        <x:v>MAT_P_TENSILE_STRENGTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B182" s="54" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C182" s="54" t="str">
+        <x:v>MAT_COMPRESSIVE</x:v>
+      </x:c>
+      <x:c r="D182" s="54" t="str">
+        <x:v>MAT_P_COMPRESSIVE_STRENGTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B183" s="54" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C183" s="54" t="str">
+        <x:v>MAT_FLEXURAL</x:v>
+      </x:c>
+      <x:c r="D183" s="54" t="str">
+        <x:v>MAT_P_FLEXURAL_STRENGTH</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B184" s="54" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C184" s="54" t="str">
+        <x:v>MAT_ELONGATION</x:v>
+      </x:c>
+      <x:c r="D184" s="54" t="str">
+        <x:v>MAT_P_ELONGATION</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B185" s="54" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C185" s="54" t="str">
+        <x:v>MAT_KIC</x:v>
+      </x:c>
+      <x:c r="D185" s="54" t="str">
+        <x:v>MAT_P_FRACTURE_TOUGHNESS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B186" s="54" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C186" s="54" t="str">
+        <x:v>MAT_THERMAL_K</x:v>
+      </x:c>
+      <x:c r="D186" s="54" t="str">
+        <x:v>MAT_P_THERMAL_CONDUCTIVITY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B187" s="54" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C187" s="54" t="str">
+        <x:v>MAT_CP</x:v>
+      </x:c>
+      <x:c r="D187" s="54" t="str">
+        <x:v>MAT_P_SPECIFIC_HEAT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B188" s="54" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C188" s="54" t="str">
+        <x:v>MAT_CTE</x:v>
+      </x:c>
+      <x:c r="D188" s="54" t="str">
+        <x:v>MAT_P_CTE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B189" s="54" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C189" s="54" t="str">
+        <x:v>MAT_RESISTIVITY</x:v>
+      </x:c>
+      <x:c r="D189" s="54" t="str">
+        <x:v>MAT_P_ELECTRICAL_RESISTIVITY</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B190" s="54" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C190" s="54" t="str">
+        <x:v>MAT_TRANSITION_T</x:v>
+      </x:c>
+      <x:c r="D190" s="54" t="str">
+        <x:v>MAT_P_TRANSITION_TEMPERATURE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B191" s="54" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C191" s="54" t="str">
+        <x:v>MAT_MAX_SERVICE_T</x:v>
+      </x:c>
+      <x:c r="D191" s="54" t="str">
+        <x:v>MAT_P_MAX_SERVICE_TEMPERATURE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B192" s="54" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="C192" s="54" t="str">
+        <x:v>MAT_HV</x:v>
+      </x:c>
+      <x:c r="D192" s="54" t="str">
+        <x:v>MAT_P_HARDNESS_VICKERS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" s="54" t="str">
+        <x:v>Property</x:v>
+      </x:c>
+      <x:c r="B193" s="54" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C193" s="54" t="str">
+        <x:v>MAT_K_BULK</x:v>
+      </x:c>
+      <x:c r="D193" s="54" t="str">
+        <x:v>MAT_P_BULK_MODULUS</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abec69a76144e7c"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -13245,7 +16206,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c41f6bba63e4a96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86fa460455a341ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13261,6 +16222,7 @@
     <x:col min="5" max="5" width="36" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="72" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="40" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -13285,6 +16247,9 @@
       <x:c r="G1" s="30" t="str">
         <x:v>Missing_Value_Behavior</x:v>
       </x:c>
+      <x:c r="H1" s="99" t="str">
+        <x:v>Materials_Source_Column</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="n">
@@ -13308,6 +16273,9 @@
       <x:c r="G2" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Density_kg_m3</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="n">
@@ -13331,6 +16299,9 @@
       <x:c r="G3" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Youngs_Modulus_GPa</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="n">
@@ -13354,6 +16325,9 @@
       <x:c r="G4" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Shear_Modulus_GPa_Derived</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="n">
@@ -13377,6 +16351,9 @@
       <x:c r="G5" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Poisson_Ratio</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="n">
@@ -13400,6 +16377,9 @@
       <x:c r="G6" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Yield_Strength_MPa</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="n">
@@ -13423,6 +16403,9 @@
       <x:c r="G7" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Tensile_Strength_MPa</x:v>
+      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="n">
@@ -13446,6 +16429,9 @@
       <x:c r="G8" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Compressive_Strength_MPa</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="n">
@@ -13469,6 +16455,9 @@
       <x:c r="G9" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Flexural_Strength_MPa</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="n">
@@ -13492,6 +16481,9 @@
       <x:c r="G10" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Elongation_Fraction</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="n">
@@ -13515,6 +16507,9 @@
       <x:c r="G11" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Fracture_Toughness_MPa_sqrt_m</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="n">
@@ -13538,6 +16533,9 @@
       <x:c r="G12" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Thermal_Conductivity_W_mK</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="n">
@@ -13561,6 +16559,9 @@
       <x:c r="G13" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Specific_Heat_J_kgK</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="n">
@@ -13584,6 +16585,9 @@
       <x:c r="G14" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H14" t="str">
+        <x:v>CTE_um_mK</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="n">
@@ -13607,6 +16611,9 @@
       <x:c r="G15" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Electrical_Resistivity_ohm_m</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="n">
@@ -13630,6 +16637,9 @@
       <x:c r="G16" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Transition_Temperature_C</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="n">
@@ -13653,6 +16663,9 @@
       <x:c r="G17" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Max_Service_Temperature_C</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="n">
@@ -13676,6 +16689,9 @@
       <x:c r="G18" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Hardness_HV</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="n">
@@ -13699,11 +16715,14 @@
       <x:c r="G19" s="7" t="str">
         <x:v>Returns DB_ERR_MISSING status and NaN value</x:v>
       </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Bulk_Modulus_GPa_Derived</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1def2fd70f3f4532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb06c03f128054268"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13926,7 +16945,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc30e301ff7834413"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0cdccff7a54434a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23589,7 +26608,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra025a0567e9044f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79233ad0e07f431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24152,4 +27171,361 @@
     </x:ext>
   </x:extLst>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="98" t="str">
+        <x:v>Key</x:v>
+      </x:c>
+      <x:c r="B1" s="98" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="C1" s="98" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="54" t="str">
+        <x:v>Dataset_ID</x:v>
+      </x:c>
+      <x:c r="B2" s="54" t="str">
+        <x:v>DRAT_ENGINEERING_MATERIALS</x:v>
+      </x:c>
+      <x:c r="C2" s="54" t="str">
+        <x:v>Stable workbook identity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="str">
+        <x:v>Schema_Version</x:v>
+      </x:c>
+      <x:c r="B3" s="54" t="str">
+        <x:v>1.0.0</x:v>
+      </x:c>
+      <x:c r="C3" s="54" t="str">
+        <x:v>Workbook contract version</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="54" t="str">
+        <x:v>Library_Name</x:v>
+      </x:c>
+      <x:c r="B4" s="54" t="str">
+        <x:v>Common Engineering Materials Library</x:v>
+      </x:c>
+      <x:c r="C4" s="54" t="str">
+        <x:v>Generated CalcPad component name</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="54" t="str">
+        <x:v>Library_Revision</x:v>
+      </x:c>
+      <x:c r="B5" s="54" t="str">
+        <x:v>1.4.0</x:v>
+      </x:c>
+      <x:c r="C5" s="54" t="str">
+        <x:v>Generated library semantic version</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="54" t="str">
+        <x:v>Library_Date</x:v>
+      </x:c>
+      <x:c r="B6" s="54" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="C6" s="54" t="str">
+        <x:v>Generated library revision date</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="54" t="str">
+        <x:v>Records_Sheet</x:v>
+      </x:c>
+      <x:c r="B7" s="54" t="str">
+        <x:v>Materials</x:v>
+      </x:c>
+      <x:c r="C7" s="54" t="str">
+        <x:v>Workbook-owned material records</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="54" t="str">
+        <x:v>Properties_Sheet</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="str">
+        <x:v>Property Dictionary</x:v>
+      </x:c>
+      <x:c r="C8" s="54" t="str">
+        <x:v>Workbook-owned property schema</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="54" t="str">
+        <x:v>Sources_Sheet</x:v>
+      </x:c>
+      <x:c r="B9" s="54" t="str">
+        <x:v>Sources</x:v>
+      </x:c>
+      <x:c r="C9" s="54" t="str">
+        <x:v>Workbook-owned source registry</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="54" t="str">
+        <x:v>Aliases_Sheet</x:v>
+      </x:c>
+      <x:c r="B10" s="54" t="str">
+        <x:v>Aliases</x:v>
+      </x:c>
+      <x:c r="C10" s="54" t="str">
+        <x:v>Workbook-owned public constant aliases</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="54" t="str">
+        <x:v>Categories_Sheet</x:v>
+      </x:c>
+      <x:c r="B11" s="54" t="str">
+        <x:v>Categories</x:v>
+      </x:c>
+      <x:c r="C11" s="54" t="str">
+        <x:v>Workbook-owned runtime category mapping</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="54" t="str">
+        <x:v>Export_Sheet</x:v>
+      </x:c>
+      <x:c r="B12" s="54" t="str">
+        <x:v>CPD Numeric Export</x:v>
+      </x:c>
+      <x:c r="C12" s="54" t="str">
+        <x:v>Auditable numeric export in property-ID order</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="54" t="str">
+        <x:v>Missing_Value</x:v>
+      </x:c>
+      <x:c r="B13" s="54" t="str">
+        <x:v>DB_MISSING</x:v>
+      </x:c>
+      <x:c r="C13" s="54" t="str">
+        <x:v>CalcPad token emitted for blank numeric cells</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Classification</x:v>
+      </x:c>
+      <x:c r="B14" s="54" t="str">
+        <x:v>MAT_CLASS_SCREENING</x:v>
+      </x:c>
+      <x:c r="C14" s="54" t="str">
+        <x:v>Current dataset classification</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="54" t="str">
+        <x:v>Data_Revision</x:v>
+      </x:c>
+      <x:c r="B15" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C15" s="54" t="str">
+        <x:v>Positive integer written to every material metadata record</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c75337caa0947de"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="98" t="str">
+        <x:v>Category_ID</x:v>
+      </x:c>
+      <x:c r="B1" s="98" t="str">
+        <x:v>CPD_Constant</x:v>
+      </x:c>
+      <x:c r="C1" s="98" t="str">
+        <x:v>Category_Name</x:v>
+      </x:c>
+      <x:c r="D1" s="98" t="str">
+        <x:v>Family</x:v>
+      </x:c>
+      <x:c r="E1" s="98" t="str">
+        <x:v>Category_Override</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="54" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="54" t="str">
+        <x:v>MAT_CAT_FERROUS_METAL</x:v>
+      </x:c>
+      <x:c r="C2" s="54" t="str">
+        <x:v>Ferrous metals</x:v>
+      </x:c>
+      <x:c r="D2" s="54" t="str">
+        <x:v>Ferrous metal</x:v>
+      </x:c>
+      <x:c r="E2" s="54" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="54" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="54" t="str">
+        <x:v>MAT_CAT_NONFERROUS_METAL</x:v>
+      </x:c>
+      <x:c r="C3" s="54" t="str">
+        <x:v>Nonferrous metals</x:v>
+      </x:c>
+      <x:c r="D3" s="54" t="str">
+        <x:v>Nonferrous metal</x:v>
+      </x:c>
+      <x:c r="E3" s="54" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="54" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="54" t="str">
+        <x:v>MAT_CAT_POLYMER</x:v>
+      </x:c>
+      <x:c r="C4" s="54" t="str">
+        <x:v>Polymers</x:v>
+      </x:c>
+      <x:c r="D4" s="54" t="str">
+        <x:v>Polymer</x:v>
+      </x:c>
+      <x:c r="E4" s="54" t="str"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="54" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="54" t="str">
+        <x:v>MAT_CAT_ELASTOMER</x:v>
+      </x:c>
+      <x:c r="C5" s="54" t="str">
+        <x:v>Elastomers</x:v>
+      </x:c>
+      <x:c r="D5" s="54" t="str">
+        <x:v>Polymer</x:v>
+      </x:c>
+      <x:c r="E5" s="54" t="str">
+        <x:v>Elastomer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="54" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="54" t="str">
+        <x:v>MAT_CAT_GLASS</x:v>
+      </x:c>
+      <x:c r="C6" s="54" t="str">
+        <x:v>Glass</x:v>
+      </x:c>
+      <x:c r="D6" s="54" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="E6" s="54" t="str">
+        <x:v>Glass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="54" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="54" t="str">
+        <x:v>MAT_CAT_CERAMIC_RELATED</x:v>
+      </x:c>
+      <x:c r="C7" s="54" t="str">
+        <x:v>Ceramics</x:v>
+      </x:c>
+      <x:c r="D7" s="54" t="str">
+        <x:v>Ceramic</x:v>
+      </x:c>
+      <x:c r="E7" s="54" t="str"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="54" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="str">
+        <x:v>MAT_CAT_COMPOSITE</x:v>
+      </x:c>
+      <x:c r="C8" s="54" t="str">
+        <x:v>Composites</x:v>
+      </x:c>
+      <x:c r="D8" s="54" t="str">
+        <x:v>Composite</x:v>
+      </x:c>
+      <x:c r="E8" s="54" t="str"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="54" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="54" t="str">
+        <x:v>MAT_CAT_WOOD</x:v>
+      </x:c>
+      <x:c r="C9" s="54" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="D9" s="54" t="str">
+        <x:v>Wood</x:v>
+      </x:c>
+      <x:c r="E9" s="54" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="54" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="54" t="str">
+        <x:v>MAT_CAT_CONSTRUCTION</x:v>
+      </x:c>
+      <x:c r="C10" s="54" t="str">
+        <x:v>Construction materials</x:v>
+      </x:c>
+      <x:c r="D10" s="54" t="str">
+        <x:v>Construction material</x:v>
+      </x:c>
+      <x:c r="E10" s="54" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228daf6105824f16"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>